<commit_message>
612 - TESTING AND TAKING SCREENSHOTS
</commit_message>
<xml_diff>
--- a/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/Network-PacketTracer/script-PACKETTRACER-IPv4.xlsx
+++ b/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/Network-PacketTracer/script-PACKETTRACER-IPv4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mannsee/Documents/Assessments/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mannsee/Documents/Assessments/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/Network-PacketTracer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAA4C8C4-9B4A-884F-96F9-423CDEA1300F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06E43E7F-19FA-1840-BC1E-54D807748973}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16580" yWindow="660" windowWidth="13660" windowHeight="18980" firstSheet="2" activeTab="7" xr2:uid="{9C60B164-F6F9-DC45-9E1B-21FD8D75857B}"/>
+    <workbookView xWindow="16580" yWindow="660" windowWidth="13660" windowHeight="18980" firstSheet="4" activeTab="7" xr2:uid="{9C60B164-F6F9-DC45-9E1B-21FD8D75857B}"/>
   </bookViews>
   <sheets>
     <sheet name="MS4-3560" sheetId="1" r:id="rId1"/>
@@ -20,8 +20,9 @@
     <sheet name="MS7-3560" sheetId="5" r:id="rId5"/>
     <sheet name="MS0-3650" sheetId="6" r:id="rId6"/>
     <sheet name="MS1-3650" sheetId="9" r:id="rId7"/>
-    <sheet name="Firewall22" sheetId="11" r:id="rId8"/>
-    <sheet name="CHECK-COMM" sheetId="10" r:id="rId9"/>
+    <sheet name="MS1-Block_Vlans" sheetId="12" r:id="rId8"/>
+    <sheet name="Firewall22" sheetId="11" r:id="rId9"/>
+    <sheet name="CHECK-COMM" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -479,11 +480,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
@@ -890,6 +891,34 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E50F22F7-84B5-DE40-B8F5-33EE5991EA40}">
+  <dimension ref="A21:A23"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="52.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="21" spans="1:1" ht="17" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59A2DE29-DDFD-084F-996E-5D8DD645CFD2}">
   <dimension ref="A1:A19"/>
@@ -1730,6 +1759,15 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{996B9398-6871-5645-A4F8-225B084F1014}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B6DA10D-BF52-0741-AE7A-9E4881301AC3}">
   <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1985,32 +2023,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E50F22F7-84B5-DE40-B8F5-33EE5991EA40}">
-  <dimension ref="A21:A23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="52.6640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="21" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>4</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
612 - added test conextoon file - arch and interfaces list
</commit_message>
<xml_diff>
--- a/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/Network-PacketTracer/script-PACKETTRACER-IPv4.xlsx
+++ b/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/Network-PacketTracer/script-PACKETTRACER-IPv4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mannsee/Documents/Assessments/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/Network-PacketTracer/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62233AB5-5E04-6641-885E-8CB850DD1DEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5209ED77-44F0-7346-A0F4-B3CAEF4F8881}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4740" yWindow="3780" windowWidth="13680" windowHeight="11480" firstSheet="4" activeTab="8" xr2:uid="{9C60B164-F6F9-DC45-9E1B-21FD8D75857B}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{9C60B164-F6F9-DC45-9E1B-21FD8D75857B}"/>
   </bookViews>
   <sheets>
     <sheet name="MS4-3560" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="123">
   <si>
     <t>enable</t>
   </si>
@@ -401,13 +401,25 @@
   </si>
   <si>
     <t xml:space="preserve"> ip access-group ACL_VLAN40 in</t>
+  </si>
+  <si>
+    <t>panning-tree portfast default</t>
+  </si>
+  <si>
+    <t>spanning-tree bpduguard default</t>
+  </si>
+  <si>
+    <t>show spanning-tree summary</t>
+  </si>
+  <si>
+    <t>spanning-tree portfast BPduguard default</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -433,6 +445,13 @@
       <color rgb="FF1F1F1F"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -541,9 +560,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -556,6 +574,12 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -870,29 +894,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B34311B4-1E30-6D40-A73D-B4C7308E242A}">
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="54.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
@@ -946,14 +970,41 @@
         <v>4</v>
       </c>
     </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="14" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>122</v>
+      </c>
+    </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A28" s="3"/>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A30" s="3"/>
+      <c r="A28" s="13"/>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A31" s="3"/>
+      <c r="A31" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -962,14 +1013,19 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E50F22F7-84B5-DE40-B8F5-33EE5991EA40}">
-  <dimension ref="A21:A23"/>
+  <dimension ref="A20:A23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="52.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="21" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="14" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
         <v>34</v>
       </c>
     </row>
@@ -990,29 +1046,29 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59A2DE29-DDFD-084F-996E-5D8DD645CFD2}">
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1063,6 +1119,39 @@
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" s="14" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="14" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="13"/>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1073,29 +1162,29 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCC59594-6BB4-1E4A-B489-1D5AC66DAC96}">
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="43.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1146,6 +1235,39 @@
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" s="14" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="14" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="13"/>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1156,129 +1278,129 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B10D8871-2FF1-AB46-91D6-9529E44202B6}">
-  <dimension ref="A1:A36"/>
+  <dimension ref="A1:A45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" s="3"/>
+      <c r="A6" s="2"/>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A10" s="3"/>
+      <c r="A10" s="2"/>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="2" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A15" s="3"/>
+      <c r="A15" s="2"/>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="2" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="2" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="2" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="2" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" s="3"/>
+      <c r="A21" s="2"/>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="2" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A23" s="3" t="s">
+      <c r="A23" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A24" s="3"/>
+      <c r="A24" s="2"/>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A26" s="4"/>
+      <c r="A26" s="3"/>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
@@ -1312,6 +1434,39 @@
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A40" s="14" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A41" s="14" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A42" s="13"/>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A45" s="2" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1322,29 +1477,29 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48880218-5589-A547-BB90-D873A156AAD1}">
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="52.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1395,6 +1550,39 @@
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="14" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="14" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" s="13"/>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1412,22 +1600,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1515,310 +1703,310 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" s="3"/>
+      <c r="A6" s="2"/>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" s="3"/>
+      <c r="A7" s="2"/>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A16" s="3"/>
+      <c r="A16" s="2"/>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" s="3"/>
+      <c r="A17" s="2"/>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" s="3"/>
+      <c r="A18" s="2"/>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A19" s="3"/>
+      <c r="A19" s="2"/>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="2" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="2" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A23" s="3"/>
+      <c r="A23" s="2"/>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="2" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="2" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="2" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A27" s="3"/>
+      <c r="A27" s="2"/>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A28" s="3" t="s">
+      <c r="A28" s="2" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A29" s="3" t="s">
+      <c r="A29" s="2" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A30" s="3" t="s">
+      <c r="A30" s="2" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A31" s="3"/>
+      <c r="A31" s="2"/>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A32" s="3" t="s">
+      <c r="A32" s="2" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A33" s="3" t="s">
+      <c r="A33" s="2" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A34" s="3" t="s">
+      <c r="A34" s="2" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A35" s="3"/>
+      <c r="A35" s="2"/>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A36" s="3"/>
+      <c r="A36" s="2"/>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A37" s="3"/>
+      <c r="A37" s="2"/>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A38" s="3"/>
+      <c r="A38" s="2"/>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A39" s="3"/>
+      <c r="A39" s="2"/>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A40" s="3" t="s">
+      <c r="A40" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A41" s="3"/>
+      <c r="A41" s="2"/>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A42" s="3" t="s">
+      <c r="A42" s="2" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A43" s="3" t="s">
+      <c r="A43" s="2" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A44" s="3"/>
+      <c r="A44" s="2"/>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A45" s="3" t="s">
+      <c r="A45" s="2" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A46" s="3" t="s">
+      <c r="A46" s="2" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A47" s="3"/>
+      <c r="A47" s="2"/>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A48" s="3" t="s">
+      <c r="A48" s="2" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A49" s="3" t="s">
+      <c r="A49" s="2" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A50" s="3"/>
+      <c r="A50" s="2"/>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A51" s="3"/>
+      <c r="A51" s="2"/>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A52" s="3"/>
+      <c r="A52" s="2"/>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A53" s="3"/>
+      <c r="A53" s="2"/>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A54" s="3" t="s">
+      <c r="A54" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A55" s="3" t="s">
+      <c r="A55" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A56" s="3"/>
+      <c r="A56" s="2"/>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A57" s="4" t="s">
+      <c r="A57" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A60" s="2" t="s">
+      <c r="A60" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A61" s="3" t="s">
+      <c r="A61" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A62" s="3" t="s">
+      <c r="A62" s="2" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A63" s="3" t="s">
+      <c r="A63" s="2" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A64" s="3" t="s">
+      <c r="A64" s="2" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A65" s="3" t="s">
+      <c r="A65" s="2" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A66" s="3" t="s">
+      <c r="A66" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A67" s="3"/>
+      <c r="A67" s="2"/>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A68" s="3" t="s">
+      <c r="A68" s="2" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A69" s="3"/>
+      <c r="A69" s="2"/>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A70" s="3" t="s">
+      <c r="A70" s="2" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A71" s="3"/>
+      <c r="A71" s="2"/>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A72" s="3" t="s">
+      <c r="A72" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A73" s="3"/>
+      <c r="A73" s="2"/>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A74" s="4" t="s">
+      <c r="A74" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1841,7 +2029,7 @@
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
@@ -2062,7 +2250,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B6DA10D-BF52-0741-AE7A-9E4881301AC3}">
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="89.6640625" customWidth="1"/>
@@ -2073,244 +2261,267 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="7" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="7" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="3"/>
-      <c r="B4" s="12" t="s">
+      <c r="A4" s="2"/>
+      <c r="B4" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="9" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="2" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="2" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="2" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" s="3"/>
+      <c r="A16" s="2"/>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" s="3"/>
+      <c r="A17" s="2"/>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" s="3"/>
+      <c r="A18" s="2"/>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="2" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" s="3"/>
+      <c r="A20" s="2"/>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="2" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A22" s="3"/>
+      <c r="A22" s="2"/>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A23" s="3"/>
+      <c r="A23" s="2"/>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="2" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="2" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A26" s="3" t="s">
+      <c r="A26" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A31" s="2" t="s">
+      <c r="A31" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A32" s="3" t="s">
+      <c r="A32" s="2" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A33" s="3" t="s">
+      <c r="A33" s="2" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A34" s="3" t="s">
+      <c r="A34" s="2" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A35" s="3" t="s">
+      <c r="A35" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A36" s="3"/>
+      <c r="A36" s="2"/>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A37" s="3" t="s">
+      <c r="A37" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A38" s="3"/>
+      <c r="A38" s="2"/>
     </row>
     <row r="39" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A39" s="13" t="s">
+      <c r="A39" s="12" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A42" s="2" t="s">
+      <c r="A42" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A44" s="1" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A43" s="3" t="s">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A45" s="2" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A44" s="3" t="s">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A46" s="2" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A45" s="3"/>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A46" s="3"/>
-    </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A47" s="3" t="s">
+      <c r="A47" s="2"/>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A48" s="2"/>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A48" s="4" t="s">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A50" s="3" t="s">
         <v>95</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A53" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A54" s="2"/>
+    </row>
+    <row r="55" spans="1:1" ht="17" x14ac:dyDescent="0.25">
+      <c r="A55" s="12" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>